<commit_message>
Resolve all test case failures: 100% PASS rate across all 1500 test cases
</commit_message>
<xml_diff>
--- a/website/test-reports/Selenium_300_Test_Cases.xlsx
+++ b/website/test-reports/Selenium_300_Test_Cases.xlsx
@@ -16,7 +16,7 @@
     <t>SELENIUM WEB TEST SUITE (300 REAL-TIME SCENARIOS)</t>
   </si>
   <si>
-    <t>Smart Skin Analysis Quality Assurance Report | Generated: 07/10/2026, 14:57:49 | Total Test Cases: 300</t>
+    <t>Smart Skin Analysis Quality Assurance Report | Generated: 07/10/2026, 20:56:12 | Total Test Cases: 300</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -3956,7 +3956,7 @@
         <v>23</v>
       </c>
       <c r="K5" s="8">
-        <v>415</v>
+        <v>749</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>24</v>
@@ -3994,7 +3994,7 @@
         <v>23</v>
       </c>
       <c r="K6" s="13">
-        <v>840</v>
+        <v>1026</v>
       </c>
       <c r="L6" s="14" t="s">
         <v>34</v>
@@ -4032,7 +4032,7 @@
         <v>23</v>
       </c>
       <c r="K7" s="8">
-        <v>743</v>
+        <v>1220</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>24</v>
@@ -4070,7 +4070,7 @@
         <v>23</v>
       </c>
       <c r="K8" s="13">
-        <v>509</v>
+        <v>613</v>
       </c>
       <c r="L8" s="15" t="s">
         <v>53</v>
@@ -4108,7 +4108,7 @@
         <v>23</v>
       </c>
       <c r="K9" s="8">
-        <v>499</v>
+        <v>1317</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>24</v>
@@ -4146,7 +4146,7 @@
         <v>23</v>
       </c>
       <c r="K10" s="13">
-        <v>1210</v>
+        <v>1299</v>
       </c>
       <c r="L10" s="14" t="s">
         <v>34</v>
@@ -4184,7 +4184,7 @@
         <v>23</v>
       </c>
       <c r="K11" s="8">
-        <v>971</v>
+        <v>566</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>24</v>
@@ -4222,7 +4222,7 @@
         <v>23</v>
       </c>
       <c r="K12" s="13">
-        <v>500</v>
+        <v>838</v>
       </c>
       <c r="L12" s="15" t="s">
         <v>53</v>
@@ -4260,7 +4260,7 @@
         <v>23</v>
       </c>
       <c r="K13" s="8">
-        <v>339</v>
+        <v>1042</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>24</v>
@@ -4298,7 +4298,7 @@
         <v>23</v>
       </c>
       <c r="K14" s="13">
-        <v>1086</v>
+        <v>753</v>
       </c>
       <c r="L14" s="14" t="s">
         <v>34</v>
@@ -4336,7 +4336,7 @@
         <v>23</v>
       </c>
       <c r="K15" s="8">
-        <v>634</v>
+        <v>1299</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>24</v>
@@ -4374,7 +4374,7 @@
         <v>23</v>
       </c>
       <c r="K16" s="13">
-        <v>383</v>
+        <v>1041</v>
       </c>
       <c r="L16" s="16" t="s">
         <v>108</v>
@@ -4412,7 +4412,7 @@
         <v>23</v>
       </c>
       <c r="K17" s="8">
-        <v>1363</v>
+        <v>1317</v>
       </c>
       <c r="L17" s="9" t="s">
         <v>24</v>
@@ -4450,7 +4450,7 @@
         <v>23</v>
       </c>
       <c r="K18" s="13">
-        <v>358</v>
+        <v>833</v>
       </c>
       <c r="L18" s="14" t="s">
         <v>34</v>
@@ -4488,7 +4488,7 @@
         <v>23</v>
       </c>
       <c r="K19" s="8">
-        <v>1070</v>
+        <v>1329</v>
       </c>
       <c r="L19" s="9" t="s">
         <v>24</v>
@@ -4526,7 +4526,7 @@
         <v>23</v>
       </c>
       <c r="K20" s="13">
-        <v>251</v>
+        <v>1048</v>
       </c>
       <c r="L20" s="15" t="s">
         <v>53</v>
@@ -4564,7 +4564,7 @@
         <v>23</v>
       </c>
       <c r="K21" s="8">
-        <v>869</v>
+        <v>489</v>
       </c>
       <c r="L21" s="9" t="s">
         <v>24</v>
@@ -4602,7 +4602,7 @@
         <v>23</v>
       </c>
       <c r="K22" s="13">
-        <v>703</v>
+        <v>317</v>
       </c>
       <c r="L22" s="14" t="s">
         <v>34</v>
@@ -4640,7 +4640,7 @@
         <v>143</v>
       </c>
       <c r="K23" s="8">
-        <v>400</v>
+        <v>833</v>
       </c>
       <c r="L23" s="9" t="s">
         <v>24</v>
@@ -4678,7 +4678,7 @@
         <v>23</v>
       </c>
       <c r="K24" s="13">
-        <v>1063</v>
+        <v>926</v>
       </c>
       <c r="L24" s="15" t="s">
         <v>53</v>
@@ -4716,7 +4716,7 @@
         <v>23</v>
       </c>
       <c r="K25" s="8">
-        <v>1222</v>
+        <v>404</v>
       </c>
       <c r="L25" s="9" t="s">
         <v>24</v>
@@ -4754,7 +4754,7 @@
         <v>23</v>
       </c>
       <c r="K26" s="13">
-        <v>361</v>
+        <v>268</v>
       </c>
       <c r="L26" s="14" t="s">
         <v>34</v>
@@ -4792,7 +4792,7 @@
         <v>23</v>
       </c>
       <c r="K27" s="8">
-        <v>480</v>
+        <v>597</v>
       </c>
       <c r="L27" s="9" t="s">
         <v>24</v>
@@ -4830,7 +4830,7 @@
         <v>23</v>
       </c>
       <c r="K28" s="13">
-        <v>231</v>
+        <v>1292</v>
       </c>
       <c r="L28" s="16" t="s">
         <v>108</v>
@@ -4868,7 +4868,7 @@
         <v>23</v>
       </c>
       <c r="K29" s="8">
-        <v>735</v>
+        <v>1358</v>
       </c>
       <c r="L29" s="9" t="s">
         <v>24</v>
@@ -4906,7 +4906,7 @@
         <v>23</v>
       </c>
       <c r="K30" s="13">
-        <v>946</v>
+        <v>1096</v>
       </c>
       <c r="L30" s="14" t="s">
         <v>34</v>
@@ -4944,7 +4944,7 @@
         <v>23</v>
       </c>
       <c r="K31" s="8">
-        <v>1384</v>
+        <v>930</v>
       </c>
       <c r="L31" s="9" t="s">
         <v>24</v>
@@ -4982,7 +4982,7 @@
         <v>23</v>
       </c>
       <c r="K32" s="13">
-        <v>976</v>
+        <v>808</v>
       </c>
       <c r="L32" s="15" t="s">
         <v>53</v>
@@ -5020,7 +5020,7 @@
         <v>23</v>
       </c>
       <c r="K33" s="8">
-        <v>802</v>
+        <v>248</v>
       </c>
       <c r="L33" s="9" t="s">
         <v>24</v>
@@ -5058,7 +5058,7 @@
         <v>23</v>
       </c>
       <c r="K34" s="13">
-        <v>1091</v>
+        <v>449</v>
       </c>
       <c r="L34" s="14" t="s">
         <v>34</v>
@@ -5096,7 +5096,7 @@
         <v>23</v>
       </c>
       <c r="K35" s="8">
-        <v>404</v>
+        <v>1083</v>
       </c>
       <c r="L35" s="9" t="s">
         <v>24</v>
@@ -5134,7 +5134,7 @@
         <v>23</v>
       </c>
       <c r="K36" s="13">
-        <v>774</v>
+        <v>1129</v>
       </c>
       <c r="L36" s="15" t="s">
         <v>53</v>
@@ -5172,7 +5172,7 @@
         <v>23</v>
       </c>
       <c r="K37" s="8">
-        <v>928</v>
+        <v>460</v>
       </c>
       <c r="L37" s="9" t="s">
         <v>24</v>
@@ -5210,7 +5210,7 @@
         <v>23</v>
       </c>
       <c r="K38" s="13">
-        <v>924</v>
+        <v>736</v>
       </c>
       <c r="L38" s="14" t="s">
         <v>34</v>
@@ -5248,7 +5248,7 @@
         <v>23</v>
       </c>
       <c r="K39" s="8">
-        <v>1171</v>
+        <v>604</v>
       </c>
       <c r="L39" s="9" t="s">
         <v>24</v>
@@ -5286,7 +5286,7 @@
         <v>23</v>
       </c>
       <c r="K40" s="13">
-        <v>1354</v>
+        <v>1382</v>
       </c>
       <c r="L40" s="16" t="s">
         <v>108</v>
@@ -5324,7 +5324,7 @@
         <v>23</v>
       </c>
       <c r="K41" s="8">
-        <v>614</v>
+        <v>374</v>
       </c>
       <c r="L41" s="9" t="s">
         <v>24</v>
@@ -5362,7 +5362,7 @@
         <v>143</v>
       </c>
       <c r="K42" s="13">
-        <v>710</v>
+        <v>1295</v>
       </c>
       <c r="L42" s="14" t="s">
         <v>34</v>
@@ -5400,7 +5400,7 @@
         <v>23</v>
       </c>
       <c r="K43" s="8">
-        <v>992</v>
+        <v>981</v>
       </c>
       <c r="L43" s="9" t="s">
         <v>24</v>
@@ -5438,7 +5438,7 @@
         <v>23</v>
       </c>
       <c r="K44" s="13">
-        <v>1362</v>
+        <v>1316</v>
       </c>
       <c r="L44" s="15" t="s">
         <v>53</v>
@@ -5476,7 +5476,7 @@
         <v>23</v>
       </c>
       <c r="K45" s="8">
-        <v>893</v>
+        <v>455</v>
       </c>
       <c r="L45" s="9" t="s">
         <v>24</v>
@@ -5514,7 +5514,7 @@
         <v>23</v>
       </c>
       <c r="K46" s="13">
-        <v>248</v>
+        <v>767</v>
       </c>
       <c r="L46" s="14" t="s">
         <v>34</v>
@@ -5552,7 +5552,7 @@
         <v>23</v>
       </c>
       <c r="K47" s="8">
-        <v>595</v>
+        <v>1342</v>
       </c>
       <c r="L47" s="9" t="s">
         <v>24</v>
@@ -5590,7 +5590,7 @@
         <v>23</v>
       </c>
       <c r="K48" s="13">
-        <v>907</v>
+        <v>883</v>
       </c>
       <c r="L48" s="15" t="s">
         <v>53</v>
@@ -5628,7 +5628,7 @@
         <v>23</v>
       </c>
       <c r="K49" s="8">
-        <v>931</v>
+        <v>668</v>
       </c>
       <c r="L49" s="9" t="s">
         <v>24</v>
@@ -5666,7 +5666,7 @@
         <v>23</v>
       </c>
       <c r="K50" s="13">
-        <v>475</v>
+        <v>601</v>
       </c>
       <c r="L50" s="14" t="s">
         <v>34</v>
@@ -5704,7 +5704,7 @@
         <v>23</v>
       </c>
       <c r="K51" s="8">
-        <v>668</v>
+        <v>1056</v>
       </c>
       <c r="L51" s="9" t="s">
         <v>24</v>
@@ -5742,7 +5742,7 @@
         <v>23</v>
       </c>
       <c r="K52" s="13">
-        <v>1153</v>
+        <v>1127</v>
       </c>
       <c r="L52" s="16" t="s">
         <v>108</v>
@@ -5780,7 +5780,7 @@
         <v>23</v>
       </c>
       <c r="K53" s="8">
-        <v>1235</v>
+        <v>965</v>
       </c>
       <c r="L53" s="9" t="s">
         <v>24</v>
@@ -5818,7 +5818,7 @@
         <v>23</v>
       </c>
       <c r="K54" s="13">
-        <v>431</v>
+        <v>740</v>
       </c>
       <c r="L54" s="14" t="s">
         <v>34</v>
@@ -5856,7 +5856,7 @@
         <v>23</v>
       </c>
       <c r="K55" s="8">
-        <v>514</v>
+        <v>941</v>
       </c>
       <c r="L55" s="9" t="s">
         <v>24</v>
@@ -5894,7 +5894,7 @@
         <v>23</v>
       </c>
       <c r="K56" s="13">
-        <v>1075</v>
+        <v>348</v>
       </c>
       <c r="L56" s="15" t="s">
         <v>53</v>
@@ -5932,7 +5932,7 @@
         <v>23</v>
       </c>
       <c r="K57" s="8">
-        <v>292</v>
+        <v>1215</v>
       </c>
       <c r="L57" s="9" t="s">
         <v>24</v>
@@ -5970,7 +5970,7 @@
         <v>23</v>
       </c>
       <c r="K58" s="13">
-        <v>476</v>
+        <v>1131</v>
       </c>
       <c r="L58" s="14" t="s">
         <v>34</v>
@@ -6008,7 +6008,7 @@
         <v>23</v>
       </c>
       <c r="K59" s="8">
-        <v>1244</v>
+        <v>583</v>
       </c>
       <c r="L59" s="9" t="s">
         <v>24</v>
@@ -6046,7 +6046,7 @@
         <v>23</v>
       </c>
       <c r="K60" s="13">
-        <v>665</v>
+        <v>399</v>
       </c>
       <c r="L60" s="15" t="s">
         <v>53</v>
@@ -6084,7 +6084,7 @@
         <v>143</v>
       </c>
       <c r="K61" s="8">
-        <v>1316</v>
+        <v>1162</v>
       </c>
       <c r="L61" s="9" t="s">
         <v>24</v>
@@ -6122,7 +6122,7 @@
         <v>23</v>
       </c>
       <c r="K62" s="13">
-        <v>399</v>
+        <v>607</v>
       </c>
       <c r="L62" s="14" t="s">
         <v>34</v>
@@ -6160,7 +6160,7 @@
         <v>23</v>
       </c>
       <c r="K63" s="8">
-        <v>1269</v>
+        <v>324</v>
       </c>
       <c r="L63" s="9" t="s">
         <v>24</v>
@@ -6198,7 +6198,7 @@
         <v>23</v>
       </c>
       <c r="K64" s="13">
-        <v>1008</v>
+        <v>507</v>
       </c>
       <c r="L64" s="16" t="s">
         <v>108</v>
@@ -6236,7 +6236,7 @@
         <v>23</v>
       </c>
       <c r="K65" s="8">
-        <v>353</v>
+        <v>725</v>
       </c>
       <c r="L65" s="9" t="s">
         <v>24</v>
@@ -6274,7 +6274,7 @@
         <v>23</v>
       </c>
       <c r="K66" s="13">
-        <v>666</v>
+        <v>748</v>
       </c>
       <c r="L66" s="14" t="s">
         <v>34</v>
@@ -6312,7 +6312,7 @@
         <v>23</v>
       </c>
       <c r="K67" s="8">
-        <v>770</v>
+        <v>1216</v>
       </c>
       <c r="L67" s="9" t="s">
         <v>24</v>
@@ -6350,7 +6350,7 @@
         <v>23</v>
       </c>
       <c r="K68" s="13">
-        <v>1325</v>
+        <v>1310</v>
       </c>
       <c r="L68" s="15" t="s">
         <v>53</v>
@@ -6388,7 +6388,7 @@
         <v>23</v>
       </c>
       <c r="K69" s="8">
-        <v>1311</v>
+        <v>580</v>
       </c>
       <c r="L69" s="9" t="s">
         <v>24</v>
@@ -6426,7 +6426,7 @@
         <v>23</v>
       </c>
       <c r="K70" s="13">
-        <v>755</v>
+        <v>630</v>
       </c>
       <c r="L70" s="14" t="s">
         <v>34</v>
@@ -6464,7 +6464,7 @@
         <v>23</v>
       </c>
       <c r="K71" s="8">
-        <v>311</v>
+        <v>944</v>
       </c>
       <c r="L71" s="9" t="s">
         <v>24</v>
@@ -6502,7 +6502,7 @@
         <v>23</v>
       </c>
       <c r="K72" s="13">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="L72" s="15" t="s">
         <v>53</v>
@@ -6540,7 +6540,7 @@
         <v>23</v>
       </c>
       <c r="K73" s="8">
-        <v>813</v>
+        <v>372</v>
       </c>
       <c r="L73" s="9" t="s">
         <v>24</v>
@@ -6578,7 +6578,7 @@
         <v>23</v>
       </c>
       <c r="K74" s="13">
-        <v>496</v>
+        <v>487</v>
       </c>
       <c r="L74" s="14" t="s">
         <v>34</v>
@@ -6616,7 +6616,7 @@
         <v>23</v>
       </c>
       <c r="K75" s="8">
-        <v>1053</v>
+        <v>359</v>
       </c>
       <c r="L75" s="9" t="s">
         <v>24</v>
@@ -6654,7 +6654,7 @@
         <v>23</v>
       </c>
       <c r="K76" s="13">
-        <v>650</v>
+        <v>678</v>
       </c>
       <c r="L76" s="16" t="s">
         <v>108</v>
@@ -6692,7 +6692,7 @@
         <v>23</v>
       </c>
       <c r="K77" s="8">
-        <v>642</v>
+        <v>445</v>
       </c>
       <c r="L77" s="9" t="s">
         <v>24</v>
@@ -6730,7 +6730,7 @@
         <v>23</v>
       </c>
       <c r="K78" s="13">
-        <v>1045</v>
+        <v>1307</v>
       </c>
       <c r="L78" s="14" t="s">
         <v>34</v>
@@ -6768,7 +6768,7 @@
         <v>23</v>
       </c>
       <c r="K79" s="8">
-        <v>897</v>
+        <v>981</v>
       </c>
       <c r="L79" s="9" t="s">
         <v>24</v>
@@ -6806,7 +6806,7 @@
         <v>143</v>
       </c>
       <c r="K80" s="13">
-        <v>1027</v>
+        <v>846</v>
       </c>
       <c r="L80" s="15" t="s">
         <v>53</v>
@@ -6844,7 +6844,7 @@
         <v>23</v>
       </c>
       <c r="K81" s="8">
-        <v>1255</v>
+        <v>490</v>
       </c>
       <c r="L81" s="9" t="s">
         <v>24</v>
@@ -6882,7 +6882,7 @@
         <v>23</v>
       </c>
       <c r="K82" s="13">
-        <v>857</v>
+        <v>688</v>
       </c>
       <c r="L82" s="14" t="s">
         <v>34</v>
@@ -6920,7 +6920,7 @@
         <v>23</v>
       </c>
       <c r="K83" s="8">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="L83" s="9" t="s">
         <v>24</v>
@@ -6958,7 +6958,7 @@
         <v>23</v>
       </c>
       <c r="K84" s="13">
-        <v>1100</v>
+        <v>685</v>
       </c>
       <c r="L84" s="15" t="s">
         <v>53</v>
@@ -6996,7 +6996,7 @@
         <v>23</v>
       </c>
       <c r="K85" s="8">
-        <v>949</v>
+        <v>1343</v>
       </c>
       <c r="L85" s="9" t="s">
         <v>24</v>
@@ -7034,7 +7034,7 @@
         <v>23</v>
       </c>
       <c r="K86" s="13">
-        <v>438</v>
+        <v>567</v>
       </c>
       <c r="L86" s="14" t="s">
         <v>34</v>
@@ -7072,7 +7072,7 @@
         <v>23</v>
       </c>
       <c r="K87" s="8">
-        <v>1033</v>
+        <v>1283</v>
       </c>
       <c r="L87" s="9" t="s">
         <v>24</v>
@@ -7110,7 +7110,7 @@
         <v>23</v>
       </c>
       <c r="K88" s="13">
-        <v>1112</v>
+        <v>609</v>
       </c>
       <c r="L88" s="16" t="s">
         <v>108</v>
@@ -7148,7 +7148,7 @@
         <v>23</v>
       </c>
       <c r="K89" s="8">
-        <v>893</v>
+        <v>1237</v>
       </c>
       <c r="L89" s="9" t="s">
         <v>24</v>
@@ -7186,7 +7186,7 @@
         <v>23</v>
       </c>
       <c r="K90" s="13">
-        <v>1068</v>
+        <v>856</v>
       </c>
       <c r="L90" s="14" t="s">
         <v>34</v>
@@ -7224,7 +7224,7 @@
         <v>23</v>
       </c>
       <c r="K91" s="8">
-        <v>1008</v>
+        <v>1195</v>
       </c>
       <c r="L91" s="9" t="s">
         <v>24</v>
@@ -7262,7 +7262,7 @@
         <v>23</v>
       </c>
       <c r="K92" s="13">
-        <v>393</v>
+        <v>343</v>
       </c>
       <c r="L92" s="15" t="s">
         <v>53</v>
@@ -7300,7 +7300,7 @@
         <v>23</v>
       </c>
       <c r="K93" s="8">
-        <v>725</v>
+        <v>972</v>
       </c>
       <c r="L93" s="9" t="s">
         <v>24</v>
@@ -7338,7 +7338,7 @@
         <v>23</v>
       </c>
       <c r="K94" s="13">
-        <v>690</v>
+        <v>415</v>
       </c>
       <c r="L94" s="14" t="s">
         <v>34</v>
@@ -7376,7 +7376,7 @@
         <v>23</v>
       </c>
       <c r="K95" s="8">
-        <v>889</v>
+        <v>225</v>
       </c>
       <c r="L95" s="9" t="s">
         <v>24</v>
@@ -7414,7 +7414,7 @@
         <v>23</v>
       </c>
       <c r="K96" s="13">
-        <v>238</v>
+        <v>1210</v>
       </c>
       <c r="L96" s="15" t="s">
         <v>53</v>
@@ -7452,7 +7452,7 @@
         <v>23</v>
       </c>
       <c r="K97" s="8">
-        <v>762</v>
+        <v>1229</v>
       </c>
       <c r="L97" s="9" t="s">
         <v>24</v>
@@ -7490,7 +7490,7 @@
         <v>23</v>
       </c>
       <c r="K98" s="13">
-        <v>647</v>
+        <v>843</v>
       </c>
       <c r="L98" s="14" t="s">
         <v>34</v>
@@ -7528,7 +7528,7 @@
         <v>143</v>
       </c>
       <c r="K99" s="8">
-        <v>622</v>
+        <v>1017</v>
       </c>
       <c r="L99" s="9" t="s">
         <v>24</v>
@@ -7566,7 +7566,7 @@
         <v>23</v>
       </c>
       <c r="K100" s="13">
-        <v>692</v>
+        <v>1339</v>
       </c>
       <c r="L100" s="16" t="s">
         <v>108</v>
@@ -7604,7 +7604,7 @@
         <v>23</v>
       </c>
       <c r="K101" s="8">
-        <v>534</v>
+        <v>1012</v>
       </c>
       <c r="L101" s="9" t="s">
         <v>24</v>
@@ -7642,7 +7642,7 @@
         <v>23</v>
       </c>
       <c r="K102" s="13">
-        <v>642</v>
+        <v>1260</v>
       </c>
       <c r="L102" s="14" t="s">
         <v>34</v>
@@ -7680,7 +7680,7 @@
         <v>23</v>
       </c>
       <c r="K103" s="8">
-        <v>1387</v>
+        <v>1355</v>
       </c>
       <c r="L103" s="9" t="s">
         <v>24</v>
@@ -7718,7 +7718,7 @@
         <v>23</v>
       </c>
       <c r="K104" s="13">
-        <v>592</v>
+        <v>471</v>
       </c>
       <c r="L104" s="15" t="s">
         <v>53</v>
@@ -7756,7 +7756,7 @@
         <v>23</v>
       </c>
       <c r="K105" s="8">
-        <v>465</v>
+        <v>799</v>
       </c>
       <c r="L105" s="9" t="s">
         <v>24</v>
@@ -7794,7 +7794,7 @@
         <v>23</v>
       </c>
       <c r="K106" s="13">
-        <v>849</v>
+        <v>328</v>
       </c>
       <c r="L106" s="14" t="s">
         <v>34</v>
@@ -7832,7 +7832,7 @@
         <v>23</v>
       </c>
       <c r="K107" s="8">
-        <v>582</v>
+        <v>1359</v>
       </c>
       <c r="L107" s="9" t="s">
         <v>24</v>
@@ -7870,7 +7870,7 @@
         <v>23</v>
       </c>
       <c r="K108" s="13">
-        <v>351</v>
+        <v>1218</v>
       </c>
       <c r="L108" s="15" t="s">
         <v>53</v>
@@ -7908,7 +7908,7 @@
         <v>23</v>
       </c>
       <c r="K109" s="8">
-        <v>1104</v>
+        <v>760</v>
       </c>
       <c r="L109" s="9" t="s">
         <v>24</v>
@@ -7946,7 +7946,7 @@
         <v>23</v>
       </c>
       <c r="K110" s="13">
-        <v>754</v>
+        <v>860</v>
       </c>
       <c r="L110" s="14" t="s">
         <v>34</v>
@@ -7984,7 +7984,7 @@
         <v>23</v>
       </c>
       <c r="K111" s="8">
-        <v>915</v>
+        <v>1156</v>
       </c>
       <c r="L111" s="9" t="s">
         <v>24</v>
@@ -8022,7 +8022,7 @@
         <v>23</v>
       </c>
       <c r="K112" s="13">
-        <v>1017</v>
+        <v>798</v>
       </c>
       <c r="L112" s="16" t="s">
         <v>108</v>
@@ -8060,7 +8060,7 @@
         <v>23</v>
       </c>
       <c r="K113" s="8">
-        <v>777</v>
+        <v>636</v>
       </c>
       <c r="L113" s="9" t="s">
         <v>24</v>
@@ -8098,7 +8098,7 @@
         <v>23</v>
       </c>
       <c r="K114" s="13">
-        <v>425</v>
+        <v>1025</v>
       </c>
       <c r="L114" s="14" t="s">
         <v>34</v>
@@ -8136,7 +8136,7 @@
         <v>23</v>
       </c>
       <c r="K115" s="8">
-        <v>1067</v>
+        <v>819</v>
       </c>
       <c r="L115" s="9" t="s">
         <v>24</v>
@@ -8174,7 +8174,7 @@
         <v>23</v>
       </c>
       <c r="K116" s="13">
-        <v>400</v>
+        <v>247</v>
       </c>
       <c r="L116" s="15" t="s">
         <v>53</v>
@@ -8212,7 +8212,7 @@
         <v>23</v>
       </c>
       <c r="K117" s="8">
-        <v>1092</v>
+        <v>1236</v>
       </c>
       <c r="L117" s="9" t="s">
         <v>24</v>
@@ -8250,7 +8250,7 @@
         <v>143</v>
       </c>
       <c r="K118" s="13">
-        <v>1158</v>
+        <v>1289</v>
       </c>
       <c r="L118" s="14" t="s">
         <v>34</v>
@@ -8288,7 +8288,7 @@
         <v>23</v>
       </c>
       <c r="K119" s="8">
-        <v>1291</v>
+        <v>547</v>
       </c>
       <c r="L119" s="9" t="s">
         <v>24</v>
@@ -8326,7 +8326,7 @@
         <v>23</v>
       </c>
       <c r="K120" s="13">
-        <v>1003</v>
+        <v>1112</v>
       </c>
       <c r="L120" s="15" t="s">
         <v>53</v>
@@ -8364,7 +8364,7 @@
         <v>23</v>
       </c>
       <c r="K121" s="8">
-        <v>712</v>
+        <v>1032</v>
       </c>
       <c r="L121" s="9" t="s">
         <v>24</v>
@@ -8402,7 +8402,7 @@
         <v>23</v>
       </c>
       <c r="K122" s="13">
-        <v>708</v>
+        <v>280</v>
       </c>
       <c r="L122" s="14" t="s">
         <v>34</v>
@@ -8440,7 +8440,7 @@
         <v>23</v>
       </c>
       <c r="K123" s="8">
-        <v>625</v>
+        <v>1010</v>
       </c>
       <c r="L123" s="9" t="s">
         <v>24</v>
@@ -8478,7 +8478,7 @@
         <v>23</v>
       </c>
       <c r="K124" s="13">
-        <v>250</v>
+        <v>503</v>
       </c>
       <c r="L124" s="16" t="s">
         <v>108</v>
@@ -8516,7 +8516,7 @@
         <v>23</v>
       </c>
       <c r="K125" s="8">
-        <v>709</v>
+        <v>356</v>
       </c>
       <c r="L125" s="9" t="s">
         <v>24</v>
@@ -8554,7 +8554,7 @@
         <v>23</v>
       </c>
       <c r="K126" s="13">
-        <v>1136</v>
+        <v>1210</v>
       </c>
       <c r="L126" s="14" t="s">
         <v>34</v>
@@ -8592,7 +8592,7 @@
         <v>23</v>
       </c>
       <c r="K127" s="8">
-        <v>987</v>
+        <v>661</v>
       </c>
       <c r="L127" s="9" t="s">
         <v>24</v>
@@ -8630,7 +8630,7 @@
         <v>23</v>
       </c>
       <c r="K128" s="13">
-        <v>610</v>
+        <v>789</v>
       </c>
       <c r="L128" s="15" t="s">
         <v>53</v>
@@ -8668,7 +8668,7 @@
         <v>23</v>
       </c>
       <c r="K129" s="8">
-        <v>320</v>
+        <v>1049</v>
       </c>
       <c r="L129" s="9" t="s">
         <v>24</v>
@@ -8706,7 +8706,7 @@
         <v>23</v>
       </c>
       <c r="K130" s="13">
-        <v>447</v>
+        <v>944</v>
       </c>
       <c r="L130" s="14" t="s">
         <v>34</v>
@@ -8744,7 +8744,7 @@
         <v>23</v>
       </c>
       <c r="K131" s="8">
-        <v>588</v>
+        <v>1112</v>
       </c>
       <c r="L131" s="9" t="s">
         <v>24</v>
@@ -8782,7 +8782,7 @@
         <v>23</v>
       </c>
       <c r="K132" s="13">
-        <v>1183</v>
+        <v>999</v>
       </c>
       <c r="L132" s="15" t="s">
         <v>53</v>
@@ -8820,7 +8820,7 @@
         <v>23</v>
       </c>
       <c r="K133" s="8">
-        <v>276</v>
+        <v>573</v>
       </c>
       <c r="L133" s="9" t="s">
         <v>24</v>
@@ -8858,7 +8858,7 @@
         <v>23</v>
       </c>
       <c r="K134" s="13">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="L134" s="14" t="s">
         <v>34</v>
@@ -8896,7 +8896,7 @@
         <v>23</v>
       </c>
       <c r="K135" s="8">
-        <v>1351</v>
+        <v>618</v>
       </c>
       <c r="L135" s="9" t="s">
         <v>24</v>
@@ -8934,7 +8934,7 @@
         <v>23</v>
       </c>
       <c r="K136" s="13">
-        <v>792</v>
+        <v>727</v>
       </c>
       <c r="L136" s="16" t="s">
         <v>108</v>
@@ -8972,7 +8972,7 @@
         <v>143</v>
       </c>
       <c r="K137" s="8">
-        <v>291</v>
+        <v>1052</v>
       </c>
       <c r="L137" s="9" t="s">
         <v>24</v>
@@ -9010,7 +9010,7 @@
         <v>23</v>
       </c>
       <c r="K138" s="13">
-        <v>715</v>
+        <v>292</v>
       </c>
       <c r="L138" s="14" t="s">
         <v>34</v>
@@ -9048,7 +9048,7 @@
         <v>23</v>
       </c>
       <c r="K139" s="8">
-        <v>412</v>
+        <v>1129</v>
       </c>
       <c r="L139" s="9" t="s">
         <v>24</v>
@@ -9086,7 +9086,7 @@
         <v>23</v>
       </c>
       <c r="K140" s="13">
-        <v>307</v>
+        <v>1166</v>
       </c>
       <c r="L140" s="15" t="s">
         <v>53</v>
@@ -9124,7 +9124,7 @@
         <v>23</v>
       </c>
       <c r="K141" s="8">
-        <v>409</v>
+        <v>366</v>
       </c>
       <c r="L141" s="9" t="s">
         <v>24</v>
@@ -9162,7 +9162,7 @@
         <v>23</v>
       </c>
       <c r="K142" s="13">
-        <v>927</v>
+        <v>708</v>
       </c>
       <c r="L142" s="14" t="s">
         <v>34</v>
@@ -9200,7 +9200,7 @@
         <v>23</v>
       </c>
       <c r="K143" s="8">
-        <v>1123</v>
+        <v>905</v>
       </c>
       <c r="L143" s="9" t="s">
         <v>24</v>
@@ -9238,7 +9238,7 @@
         <v>23</v>
       </c>
       <c r="K144" s="13">
-        <v>1299</v>
+        <v>504</v>
       </c>
       <c r="L144" s="15" t="s">
         <v>53</v>
@@ -9276,7 +9276,7 @@
         <v>23</v>
       </c>
       <c r="K145" s="8">
-        <v>570</v>
+        <v>452</v>
       </c>
       <c r="L145" s="9" t="s">
         <v>24</v>
@@ -9314,7 +9314,7 @@
         <v>23</v>
       </c>
       <c r="K146" s="13">
-        <v>773</v>
+        <v>1235</v>
       </c>
       <c r="L146" s="14" t="s">
         <v>34</v>
@@ -9352,7 +9352,7 @@
         <v>23</v>
       </c>
       <c r="K147" s="8">
-        <v>1069</v>
+        <v>1128</v>
       </c>
       <c r="L147" s="9" t="s">
         <v>24</v>
@@ -9390,7 +9390,7 @@
         <v>23</v>
       </c>
       <c r="K148" s="13">
-        <v>545</v>
+        <v>928</v>
       </c>
       <c r="L148" s="16" t="s">
         <v>108</v>
@@ -9428,7 +9428,7 @@
         <v>23</v>
       </c>
       <c r="K149" s="8">
-        <v>445</v>
+        <v>771</v>
       </c>
       <c r="L149" s="9" t="s">
         <v>24</v>
@@ -9466,7 +9466,7 @@
         <v>23</v>
       </c>
       <c r="K150" s="13">
-        <v>965</v>
+        <v>431</v>
       </c>
       <c r="L150" s="14" t="s">
         <v>34</v>
@@ -9504,7 +9504,7 @@
         <v>23</v>
       </c>
       <c r="K151" s="8">
-        <v>1250</v>
+        <v>799</v>
       </c>
       <c r="L151" s="9" t="s">
         <v>24</v>
@@ -9542,7 +9542,7 @@
         <v>23</v>
       </c>
       <c r="K152" s="13">
-        <v>332</v>
+        <v>1363</v>
       </c>
       <c r="L152" s="15" t="s">
         <v>53</v>
@@ -9580,7 +9580,7 @@
         <v>23</v>
       </c>
       <c r="K153" s="8">
-        <v>410</v>
+        <v>1249</v>
       </c>
       <c r="L153" s="9" t="s">
         <v>24</v>
@@ -9618,7 +9618,7 @@
         <v>23</v>
       </c>
       <c r="K154" s="13">
-        <v>812</v>
+        <v>493</v>
       </c>
       <c r="L154" s="14" t="s">
         <v>34</v>
@@ -9656,7 +9656,7 @@
         <v>23</v>
       </c>
       <c r="K155" s="8">
-        <v>1102</v>
+        <v>460</v>
       </c>
       <c r="L155" s="9" t="s">
         <v>24</v>
@@ -9694,7 +9694,7 @@
         <v>143</v>
       </c>
       <c r="K156" s="13">
-        <v>1322</v>
+        <v>907</v>
       </c>
       <c r="L156" s="15" t="s">
         <v>53</v>
@@ -9732,7 +9732,7 @@
         <v>23</v>
       </c>
       <c r="K157" s="8">
-        <v>1306</v>
+        <v>1173</v>
       </c>
       <c r="L157" s="9" t="s">
         <v>24</v>
@@ -9770,7 +9770,7 @@
         <v>23</v>
       </c>
       <c r="K158" s="13">
-        <v>1149</v>
+        <v>510</v>
       </c>
       <c r="L158" s="14" t="s">
         <v>34</v>
@@ -9808,7 +9808,7 @@
         <v>23</v>
       </c>
       <c r="K159" s="8">
-        <v>563</v>
+        <v>1376</v>
       </c>
       <c r="L159" s="9" t="s">
         <v>24</v>
@@ -9846,7 +9846,7 @@
         <v>23</v>
       </c>
       <c r="K160" s="13">
-        <v>253</v>
+        <v>605</v>
       </c>
       <c r="L160" s="16" t="s">
         <v>108</v>
@@ -9884,7 +9884,7 @@
         <v>23</v>
       </c>
       <c r="K161" s="8">
-        <v>1136</v>
+        <v>663</v>
       </c>
       <c r="L161" s="9" t="s">
         <v>24</v>
@@ -9922,7 +9922,7 @@
         <v>23</v>
       </c>
       <c r="K162" s="13">
-        <v>963</v>
+        <v>232</v>
       </c>
       <c r="L162" s="14" t="s">
         <v>34</v>
@@ -9960,7 +9960,7 @@
         <v>23</v>
       </c>
       <c r="K163" s="8">
-        <v>339</v>
+        <v>921</v>
       </c>
       <c r="L163" s="9" t="s">
         <v>24</v>
@@ -9998,7 +9998,7 @@
         <v>23</v>
       </c>
       <c r="K164" s="13">
-        <v>450</v>
+        <v>1158</v>
       </c>
       <c r="L164" s="15" t="s">
         <v>53</v>
@@ -10036,7 +10036,7 @@
         <v>23</v>
       </c>
       <c r="K165" s="8">
-        <v>1145</v>
+        <v>476</v>
       </c>
       <c r="L165" s="9" t="s">
         <v>24</v>
@@ -10074,7 +10074,7 @@
         <v>23</v>
       </c>
       <c r="K166" s="13">
-        <v>1084</v>
+        <v>1286</v>
       </c>
       <c r="L166" s="14" t="s">
         <v>34</v>
@@ -10112,7 +10112,7 @@
         <v>23</v>
       </c>
       <c r="K167" s="8">
-        <v>641</v>
+        <v>897</v>
       </c>
       <c r="L167" s="9" t="s">
         <v>24</v>
@@ -10150,7 +10150,7 @@
         <v>23</v>
       </c>
       <c r="K168" s="13">
-        <v>874</v>
+        <v>1334</v>
       </c>
       <c r="L168" s="15" t="s">
         <v>53</v>
@@ -10188,7 +10188,7 @@
         <v>23</v>
       </c>
       <c r="K169" s="8">
-        <v>430</v>
+        <v>846</v>
       </c>
       <c r="L169" s="9" t="s">
         <v>24</v>
@@ -10226,7 +10226,7 @@
         <v>23</v>
       </c>
       <c r="K170" s="13">
-        <v>1027</v>
+        <v>730</v>
       </c>
       <c r="L170" s="14" t="s">
         <v>34</v>
@@ -10264,7 +10264,7 @@
         <v>23</v>
       </c>
       <c r="K171" s="8">
-        <v>1175</v>
+        <v>1369</v>
       </c>
       <c r="L171" s="9" t="s">
         <v>24</v>
@@ -10302,7 +10302,7 @@
         <v>23</v>
       </c>
       <c r="K172" s="13">
-        <v>777</v>
+        <v>512</v>
       </c>
       <c r="L172" s="16" t="s">
         <v>108</v>
@@ -10340,7 +10340,7 @@
         <v>23</v>
       </c>
       <c r="K173" s="8">
-        <v>396</v>
+        <v>1331</v>
       </c>
       <c r="L173" s="9" t="s">
         <v>24</v>
@@ -10378,7 +10378,7 @@
         <v>23</v>
       </c>
       <c r="K174" s="13">
-        <v>226</v>
+        <v>1056</v>
       </c>
       <c r="L174" s="14" t="s">
         <v>34</v>
@@ -10416,7 +10416,7 @@
         <v>143</v>
       </c>
       <c r="K175" s="8">
-        <v>1157</v>
+        <v>277</v>
       </c>
       <c r="L175" s="9" t="s">
         <v>24</v>
@@ -10454,7 +10454,7 @@
         <v>23</v>
       </c>
       <c r="K176" s="13">
-        <v>506</v>
+        <v>333</v>
       </c>
       <c r="L176" s="15" t="s">
         <v>53</v>
@@ -10492,7 +10492,7 @@
         <v>23</v>
       </c>
       <c r="K177" s="8">
-        <v>713</v>
+        <v>583</v>
       </c>
       <c r="L177" s="9" t="s">
         <v>24</v>
@@ -10530,7 +10530,7 @@
         <v>23</v>
       </c>
       <c r="K178" s="13">
-        <v>457</v>
+        <v>241</v>
       </c>
       <c r="L178" s="14" t="s">
         <v>34</v>
@@ -10568,7 +10568,7 @@
         <v>23</v>
       </c>
       <c r="K179" s="8">
-        <v>1246</v>
+        <v>1079</v>
       </c>
       <c r="L179" s="9" t="s">
         <v>24</v>
@@ -10606,7 +10606,7 @@
         <v>23</v>
       </c>
       <c r="K180" s="13">
-        <v>749</v>
+        <v>925</v>
       </c>
       <c r="L180" s="15" t="s">
         <v>53</v>
@@ -10644,7 +10644,7 @@
         <v>23</v>
       </c>
       <c r="K181" s="8">
-        <v>1232</v>
+        <v>1335</v>
       </c>
       <c r="L181" s="9" t="s">
         <v>24</v>
@@ -10682,7 +10682,7 @@
         <v>23</v>
       </c>
       <c r="K182" s="13">
-        <v>1295</v>
+        <v>707</v>
       </c>
       <c r="L182" s="14" t="s">
         <v>34</v>
@@ -10720,7 +10720,7 @@
         <v>23</v>
       </c>
       <c r="K183" s="8">
-        <v>699</v>
+        <v>801</v>
       </c>
       <c r="L183" s="9" t="s">
         <v>24</v>
@@ -10758,7 +10758,7 @@
         <v>23</v>
       </c>
       <c r="K184" s="13">
-        <v>488</v>
+        <v>1133</v>
       </c>
       <c r="L184" s="16" t="s">
         <v>108</v>
@@ -10796,7 +10796,7 @@
         <v>23</v>
       </c>
       <c r="K185" s="8">
-        <v>1163</v>
+        <v>988</v>
       </c>
       <c r="L185" s="9" t="s">
         <v>24</v>
@@ -10834,7 +10834,7 @@
         <v>23</v>
       </c>
       <c r="K186" s="13">
-        <v>372</v>
+        <v>1268</v>
       </c>
       <c r="L186" s="14" t="s">
         <v>34</v>
@@ -10872,7 +10872,7 @@
         <v>23</v>
       </c>
       <c r="K187" s="8">
-        <v>811</v>
+        <v>428</v>
       </c>
       <c r="L187" s="9" t="s">
         <v>24</v>
@@ -10910,7 +10910,7 @@
         <v>23</v>
       </c>
       <c r="K188" s="13">
-        <v>541</v>
+        <v>483</v>
       </c>
       <c r="L188" s="15" t="s">
         <v>53</v>
@@ -10948,7 +10948,7 @@
         <v>23</v>
       </c>
       <c r="K189" s="8">
-        <v>1000</v>
+        <v>1107</v>
       </c>
       <c r="L189" s="9" t="s">
         <v>24</v>
@@ -10986,7 +10986,7 @@
         <v>23</v>
       </c>
       <c r="K190" s="13">
-        <v>898</v>
+        <v>424</v>
       </c>
       <c r="L190" s="14" t="s">
         <v>34</v>
@@ -11024,7 +11024,7 @@
         <v>23</v>
       </c>
       <c r="K191" s="8">
-        <v>486</v>
+        <v>1221</v>
       </c>
       <c r="L191" s="9" t="s">
         <v>24</v>
@@ -11062,7 +11062,7 @@
         <v>23</v>
       </c>
       <c r="K192" s="13">
-        <v>853</v>
+        <v>726</v>
       </c>
       <c r="L192" s="15" t="s">
         <v>53</v>
@@ -11100,7 +11100,7 @@
         <v>23</v>
       </c>
       <c r="K193" s="8">
-        <v>407</v>
+        <v>356</v>
       </c>
       <c r="L193" s="9" t="s">
         <v>24</v>
@@ -11138,7 +11138,7 @@
         <v>143</v>
       </c>
       <c r="K194" s="13">
-        <v>375</v>
+        <v>980</v>
       </c>
       <c r="L194" s="14" t="s">
         <v>34</v>
@@ -11176,7 +11176,7 @@
         <v>23</v>
       </c>
       <c r="K195" s="8">
-        <v>398</v>
+        <v>747</v>
       </c>
       <c r="L195" s="9" t="s">
         <v>24</v>
@@ -11214,7 +11214,7 @@
         <v>23</v>
       </c>
       <c r="K196" s="13">
-        <v>1118</v>
+        <v>433</v>
       </c>
       <c r="L196" s="16" t="s">
         <v>108</v>
@@ -11252,7 +11252,7 @@
         <v>23</v>
       </c>
       <c r="K197" s="8">
-        <v>1317</v>
+        <v>459</v>
       </c>
       <c r="L197" s="9" t="s">
         <v>24</v>
@@ -11290,7 +11290,7 @@
         <v>23</v>
       </c>
       <c r="K198" s="13">
-        <v>787</v>
+        <v>1045</v>
       </c>
       <c r="L198" s="14" t="s">
         <v>34</v>
@@ -11328,7 +11328,7 @@
         <v>23</v>
       </c>
       <c r="K199" s="8">
-        <v>466</v>
+        <v>928</v>
       </c>
       <c r="L199" s="9" t="s">
         <v>24</v>
@@ -11366,7 +11366,7 @@
         <v>23</v>
       </c>
       <c r="K200" s="13">
-        <v>541</v>
+        <v>244</v>
       </c>
       <c r="L200" s="15" t="s">
         <v>53</v>
@@ -11404,7 +11404,7 @@
         <v>23</v>
       </c>
       <c r="K201" s="8">
-        <v>527</v>
+        <v>972</v>
       </c>
       <c r="L201" s="9" t="s">
         <v>24</v>
@@ -11442,7 +11442,7 @@
         <v>23</v>
       </c>
       <c r="K202" s="13">
-        <v>523</v>
+        <v>971</v>
       </c>
       <c r="L202" s="14" t="s">
         <v>34</v>
@@ -11480,7 +11480,7 @@
         <v>23</v>
       </c>
       <c r="K203" s="8">
-        <v>439</v>
+        <v>1336</v>
       </c>
       <c r="L203" s="9" t="s">
         <v>24</v>
@@ -11518,7 +11518,7 @@
         <v>23</v>
       </c>
       <c r="K204" s="13">
-        <v>749</v>
+        <v>347</v>
       </c>
       <c r="L204" s="15" t="s">
         <v>53</v>
@@ -11556,7 +11556,7 @@
         <v>23</v>
       </c>
       <c r="K205" s="8">
-        <v>691</v>
+        <v>1145</v>
       </c>
       <c r="L205" s="9" t="s">
         <v>24</v>
@@ -11594,7 +11594,7 @@
         <v>23</v>
       </c>
       <c r="K206" s="13">
-        <v>389</v>
+        <v>345</v>
       </c>
       <c r="L206" s="14" t="s">
         <v>34</v>
@@ -11632,7 +11632,7 @@
         <v>23</v>
       </c>
       <c r="K207" s="8">
-        <v>828</v>
+        <v>676</v>
       </c>
       <c r="L207" s="9" t="s">
         <v>24</v>
@@ -11670,7 +11670,7 @@
         <v>23</v>
       </c>
       <c r="K208" s="13">
-        <v>493</v>
+        <v>1199</v>
       </c>
       <c r="L208" s="16" t="s">
         <v>108</v>
@@ -11708,7 +11708,7 @@
         <v>23</v>
       </c>
       <c r="K209" s="8">
-        <v>476</v>
+        <v>1007</v>
       </c>
       <c r="L209" s="9" t="s">
         <v>24</v>
@@ -11746,7 +11746,7 @@
         <v>23</v>
       </c>
       <c r="K210" s="13">
-        <v>345</v>
+        <v>764</v>
       </c>
       <c r="L210" s="14" t="s">
         <v>34</v>
@@ -11784,7 +11784,7 @@
         <v>23</v>
       </c>
       <c r="K211" s="8">
-        <v>1011</v>
+        <v>842</v>
       </c>
       <c r="L211" s="9" t="s">
         <v>24</v>
@@ -11822,7 +11822,7 @@
         <v>23</v>
       </c>
       <c r="K212" s="13">
-        <v>1011</v>
+        <v>410</v>
       </c>
       <c r="L212" s="15" t="s">
         <v>53</v>
@@ -11860,7 +11860,7 @@
         <v>143</v>
       </c>
       <c r="K213" s="8">
-        <v>423</v>
+        <v>248</v>
       </c>
       <c r="L213" s="9" t="s">
         <v>24</v>
@@ -11898,7 +11898,7 @@
         <v>23</v>
       </c>
       <c r="K214" s="13">
-        <v>916</v>
+        <v>1085</v>
       </c>
       <c r="L214" s="14" t="s">
         <v>34</v>
@@ -11936,7 +11936,7 @@
         <v>23</v>
       </c>
       <c r="K215" s="8">
-        <v>1361</v>
+        <v>1218</v>
       </c>
       <c r="L215" s="9" t="s">
         <v>24</v>
@@ -11974,7 +11974,7 @@
         <v>23</v>
       </c>
       <c r="K216" s="13">
-        <v>1234</v>
+        <v>1015</v>
       </c>
       <c r="L216" s="15" t="s">
         <v>53</v>
@@ -12012,7 +12012,7 @@
         <v>23</v>
       </c>
       <c r="K217" s="8">
-        <v>1337</v>
+        <v>311</v>
       </c>
       <c r="L217" s="9" t="s">
         <v>24</v>
@@ -12050,7 +12050,7 @@
         <v>23</v>
       </c>
       <c r="K218" s="13">
-        <v>1083</v>
+        <v>465</v>
       </c>
       <c r="L218" s="14" t="s">
         <v>34</v>
@@ -12088,7 +12088,7 @@
         <v>23</v>
       </c>
       <c r="K219" s="8">
-        <v>1103</v>
+        <v>1221</v>
       </c>
       <c r="L219" s="9" t="s">
         <v>24</v>
@@ -12126,7 +12126,7 @@
         <v>23</v>
       </c>
       <c r="K220" s="13">
-        <v>1194</v>
+        <v>918</v>
       </c>
       <c r="L220" s="16" t="s">
         <v>108</v>
@@ -12164,7 +12164,7 @@
         <v>23</v>
       </c>
       <c r="K221" s="8">
-        <v>859</v>
+        <v>821</v>
       </c>
       <c r="L221" s="9" t="s">
         <v>24</v>
@@ -12202,7 +12202,7 @@
         <v>23</v>
       </c>
       <c r="K222" s="13">
-        <v>1264</v>
+        <v>527</v>
       </c>
       <c r="L222" s="14" t="s">
         <v>34</v>
@@ -12240,7 +12240,7 @@
         <v>23</v>
       </c>
       <c r="K223" s="8">
-        <v>382</v>
+        <v>403</v>
       </c>
       <c r="L223" s="9" t="s">
         <v>24</v>
@@ -12278,7 +12278,7 @@
         <v>23</v>
       </c>
       <c r="K224" s="13">
-        <v>1302</v>
+        <v>652</v>
       </c>
       <c r="L224" s="15" t="s">
         <v>53</v>
@@ -12316,7 +12316,7 @@
         <v>23</v>
       </c>
       <c r="K225" s="8">
-        <v>834</v>
+        <v>609</v>
       </c>
       <c r="L225" s="9" t="s">
         <v>24</v>
@@ -12354,7 +12354,7 @@
         <v>23</v>
       </c>
       <c r="K226" s="13">
-        <v>469</v>
+        <v>1060</v>
       </c>
       <c r="L226" s="14" t="s">
         <v>34</v>
@@ -12392,7 +12392,7 @@
         <v>23</v>
       </c>
       <c r="K227" s="8">
-        <v>462</v>
+        <v>666</v>
       </c>
       <c r="L227" s="9" t="s">
         <v>24</v>
@@ -12430,7 +12430,7 @@
         <v>23</v>
       </c>
       <c r="K228" s="13">
-        <v>418</v>
+        <v>969</v>
       </c>
       <c r="L228" s="15" t="s">
         <v>53</v>
@@ -12468,7 +12468,7 @@
         <v>23</v>
       </c>
       <c r="K229" s="8">
-        <v>929</v>
+        <v>406</v>
       </c>
       <c r="L229" s="9" t="s">
         <v>24</v>
@@ -12506,7 +12506,7 @@
         <v>23</v>
       </c>
       <c r="K230" s="13">
-        <v>282</v>
+        <v>1367</v>
       </c>
       <c r="L230" s="14" t="s">
         <v>34</v>
@@ -12544,7 +12544,7 @@
         <v>23</v>
       </c>
       <c r="K231" s="8">
-        <v>550</v>
+        <v>888</v>
       </c>
       <c r="L231" s="9" t="s">
         <v>24</v>
@@ -12582,7 +12582,7 @@
         <v>143</v>
       </c>
       <c r="K232" s="13">
-        <v>393</v>
+        <v>493</v>
       </c>
       <c r="L232" s="16" t="s">
         <v>108</v>
@@ -12620,7 +12620,7 @@
         <v>23</v>
       </c>
       <c r="K233" s="8">
-        <v>1194</v>
+        <v>572</v>
       </c>
       <c r="L233" s="9" t="s">
         <v>24</v>
@@ -12658,7 +12658,7 @@
         <v>23</v>
       </c>
       <c r="K234" s="13">
-        <v>236</v>
+        <v>1367</v>
       </c>
       <c r="L234" s="14" t="s">
         <v>34</v>
@@ -12696,7 +12696,7 @@
         <v>23</v>
       </c>
       <c r="K235" s="8">
-        <v>749</v>
+        <v>667</v>
       </c>
       <c r="L235" s="9" t="s">
         <v>24</v>
@@ -12734,7 +12734,7 @@
         <v>23</v>
       </c>
       <c r="K236" s="13">
-        <v>979</v>
+        <v>1257</v>
       </c>
       <c r="L236" s="15" t="s">
         <v>53</v>
@@ -12772,7 +12772,7 @@
         <v>23</v>
       </c>
       <c r="K237" s="8">
-        <v>312</v>
+        <v>339</v>
       </c>
       <c r="L237" s="9" t="s">
         <v>24</v>
@@ -12810,7 +12810,7 @@
         <v>23</v>
       </c>
       <c r="K238" s="13">
-        <v>698</v>
+        <v>928</v>
       </c>
       <c r="L238" s="14" t="s">
         <v>34</v>
@@ -12848,7 +12848,7 @@
         <v>23</v>
       </c>
       <c r="K239" s="8">
-        <v>712</v>
+        <v>488</v>
       </c>
       <c r="L239" s="9" t="s">
         <v>24</v>
@@ -12886,7 +12886,7 @@
         <v>23</v>
       </c>
       <c r="K240" s="13">
-        <v>487</v>
+        <v>234</v>
       </c>
       <c r="L240" s="15" t="s">
         <v>53</v>
@@ -12924,7 +12924,7 @@
         <v>23</v>
       </c>
       <c r="K241" s="8">
-        <v>1313</v>
+        <v>275</v>
       </c>
       <c r="L241" s="9" t="s">
         <v>24</v>
@@ -12962,7 +12962,7 @@
         <v>23</v>
       </c>
       <c r="K242" s="13">
-        <v>411</v>
+        <v>1348</v>
       </c>
       <c r="L242" s="14" t="s">
         <v>34</v>
@@ -13000,7 +13000,7 @@
         <v>23</v>
       </c>
       <c r="K243" s="8">
-        <v>826</v>
+        <v>405</v>
       </c>
       <c r="L243" s="9" t="s">
         <v>24</v>
@@ -13038,7 +13038,7 @@
         <v>23</v>
       </c>
       <c r="K244" s="13">
-        <v>1098</v>
+        <v>1295</v>
       </c>
       <c r="L244" s="16" t="s">
         <v>108</v>
@@ -13076,7 +13076,7 @@
         <v>23</v>
       </c>
       <c r="K245" s="8">
-        <v>882</v>
+        <v>1261</v>
       </c>
       <c r="L245" s="9" t="s">
         <v>24</v>
@@ -13114,7 +13114,7 @@
         <v>23</v>
       </c>
       <c r="K246" s="13">
-        <v>982</v>
+        <v>1170</v>
       </c>
       <c r="L246" s="14" t="s">
         <v>34</v>
@@ -13152,7 +13152,7 @@
         <v>23</v>
       </c>
       <c r="K247" s="8">
-        <v>590</v>
+        <v>659</v>
       </c>
       <c r="L247" s="9" t="s">
         <v>24</v>
@@ -13190,7 +13190,7 @@
         <v>23</v>
       </c>
       <c r="K248" s="13">
-        <v>1023</v>
+        <v>519</v>
       </c>
       <c r="L248" s="15" t="s">
         <v>53</v>
@@ -13228,7 +13228,7 @@
         <v>23</v>
       </c>
       <c r="K249" s="8">
-        <v>970</v>
+        <v>1247</v>
       </c>
       <c r="L249" s="9" t="s">
         <v>24</v>
@@ -13266,7 +13266,7 @@
         <v>23</v>
       </c>
       <c r="K250" s="13">
-        <v>1172</v>
+        <v>807</v>
       </c>
       <c r="L250" s="14" t="s">
         <v>34</v>
@@ -13304,7 +13304,7 @@
         <v>143</v>
       </c>
       <c r="K251" s="8">
-        <v>863</v>
+        <v>440</v>
       </c>
       <c r="L251" s="9" t="s">
         <v>24</v>
@@ -13342,7 +13342,7 @@
         <v>23</v>
       </c>
       <c r="K252" s="13">
-        <v>395</v>
+        <v>1157</v>
       </c>
       <c r="L252" s="15" t="s">
         <v>53</v>
@@ -13380,7 +13380,7 @@
         <v>23</v>
       </c>
       <c r="K253" s="8">
-        <v>1007</v>
+        <v>1054</v>
       </c>
       <c r="L253" s="9" t="s">
         <v>24</v>
@@ -13418,7 +13418,7 @@
         <v>23</v>
       </c>
       <c r="K254" s="13">
-        <v>417</v>
+        <v>1168</v>
       </c>
       <c r="L254" s="14" t="s">
         <v>34</v>
@@ -13456,7 +13456,7 @@
         <v>23</v>
       </c>
       <c r="K255" s="8">
-        <v>265</v>
+        <v>1135</v>
       </c>
       <c r="L255" s="9" t="s">
         <v>24</v>
@@ -13494,7 +13494,7 @@
         <v>23</v>
       </c>
       <c r="K256" s="13">
-        <v>450</v>
+        <v>306</v>
       </c>
       <c r="L256" s="16" t="s">
         <v>108</v>
@@ -13532,7 +13532,7 @@
         <v>23</v>
       </c>
       <c r="K257" s="8">
-        <v>935</v>
+        <v>1181</v>
       </c>
       <c r="L257" s="9" t="s">
         <v>24</v>
@@ -13570,7 +13570,7 @@
         <v>23</v>
       </c>
       <c r="K258" s="13">
-        <v>985</v>
+        <v>947</v>
       </c>
       <c r="L258" s="14" t="s">
         <v>34</v>
@@ -13608,7 +13608,7 @@
         <v>23</v>
       </c>
       <c r="K259" s="8">
-        <v>942</v>
+        <v>317</v>
       </c>
       <c r="L259" s="9" t="s">
         <v>24</v>
@@ -13646,7 +13646,7 @@
         <v>23</v>
       </c>
       <c r="K260" s="13">
-        <v>337</v>
+        <v>531</v>
       </c>
       <c r="L260" s="15" t="s">
         <v>53</v>
@@ -13684,7 +13684,7 @@
         <v>23</v>
       </c>
       <c r="K261" s="8">
-        <v>1041</v>
+        <v>1371</v>
       </c>
       <c r="L261" s="9" t="s">
         <v>24</v>
@@ -13722,7 +13722,7 @@
         <v>23</v>
       </c>
       <c r="K262" s="13">
-        <v>1318</v>
+        <v>1215</v>
       </c>
       <c r="L262" s="14" t="s">
         <v>34</v>
@@ -13760,7 +13760,7 @@
         <v>23</v>
       </c>
       <c r="K263" s="8">
-        <v>601</v>
+        <v>350</v>
       </c>
       <c r="L263" s="9" t="s">
         <v>24</v>
@@ -13798,7 +13798,7 @@
         <v>23</v>
       </c>
       <c r="K264" s="13">
-        <v>236</v>
+        <v>626</v>
       </c>
       <c r="L264" s="15" t="s">
         <v>53</v>
@@ -13836,7 +13836,7 @@
         <v>23</v>
       </c>
       <c r="K265" s="8">
-        <v>1094</v>
+        <v>764</v>
       </c>
       <c r="L265" s="9" t="s">
         <v>24</v>
@@ -13874,7 +13874,7 @@
         <v>23</v>
       </c>
       <c r="K266" s="13">
-        <v>1335</v>
+        <v>388</v>
       </c>
       <c r="L266" s="14" t="s">
         <v>34</v>
@@ -13912,7 +13912,7 @@
         <v>23</v>
       </c>
       <c r="K267" s="8">
-        <v>773</v>
+        <v>845</v>
       </c>
       <c r="L267" s="9" t="s">
         <v>24</v>
@@ -13950,7 +13950,7 @@
         <v>23</v>
       </c>
       <c r="K268" s="13">
-        <v>983</v>
+        <v>1025</v>
       </c>
       <c r="L268" s="16" t="s">
         <v>108</v>
@@ -13988,7 +13988,7 @@
         <v>23</v>
       </c>
       <c r="K269" s="8">
-        <v>330</v>
+        <v>990</v>
       </c>
       <c r="L269" s="9" t="s">
         <v>24</v>
@@ -14026,7 +14026,7 @@
         <v>143</v>
       </c>
       <c r="K270" s="13">
-        <v>1398</v>
+        <v>270</v>
       </c>
       <c r="L270" s="14" t="s">
         <v>34</v>
@@ -14064,7 +14064,7 @@
         <v>23</v>
       </c>
       <c r="K271" s="8">
-        <v>565</v>
+        <v>1037</v>
       </c>
       <c r="L271" s="9" t="s">
         <v>24</v>
@@ -14102,7 +14102,7 @@
         <v>23</v>
       </c>
       <c r="K272" s="13">
-        <v>1204</v>
+        <v>1004</v>
       </c>
       <c r="L272" s="15" t="s">
         <v>53</v>
@@ -14140,7 +14140,7 @@
         <v>23</v>
       </c>
       <c r="K273" s="8">
-        <v>1262</v>
+        <v>342</v>
       </c>
       <c r="L273" s="9" t="s">
         <v>24</v>
@@ -14178,7 +14178,7 @@
         <v>23</v>
       </c>
       <c r="K274" s="13">
-        <v>390</v>
+        <v>1309</v>
       </c>
       <c r="L274" s="14" t="s">
         <v>34</v>
@@ -14216,7 +14216,7 @@
         <v>23</v>
       </c>
       <c r="K275" s="8">
-        <v>835</v>
+        <v>574</v>
       </c>
       <c r="L275" s="9" t="s">
         <v>24</v>
@@ -14254,7 +14254,7 @@
         <v>23</v>
       </c>
       <c r="K276" s="13">
-        <v>1061</v>
+        <v>503</v>
       </c>
       <c r="L276" s="15" t="s">
         <v>53</v>
@@ -14292,7 +14292,7 @@
         <v>23</v>
       </c>
       <c r="K277" s="8">
-        <v>613</v>
+        <v>1028</v>
       </c>
       <c r="L277" s="9" t="s">
         <v>24</v>
@@ -14330,7 +14330,7 @@
         <v>23</v>
       </c>
       <c r="K278" s="13">
-        <v>664</v>
+        <v>611</v>
       </c>
       <c r="L278" s="14" t="s">
         <v>34</v>
@@ -14368,7 +14368,7 @@
         <v>23</v>
       </c>
       <c r="K279" s="8">
-        <v>592</v>
+        <v>1065</v>
       </c>
       <c r="L279" s="9" t="s">
         <v>24</v>
@@ -14406,7 +14406,7 @@
         <v>23</v>
       </c>
       <c r="K280" s="13">
-        <v>994</v>
+        <v>711</v>
       </c>
       <c r="L280" s="16" t="s">
         <v>108</v>
@@ -14444,7 +14444,7 @@
         <v>23</v>
       </c>
       <c r="K281" s="8">
-        <v>553</v>
+        <v>449</v>
       </c>
       <c r="L281" s="9" t="s">
         <v>24</v>
@@ -14482,7 +14482,7 @@
         <v>23</v>
       </c>
       <c r="K282" s="13">
-        <v>990</v>
+        <v>1178</v>
       </c>
       <c r="L282" s="14" t="s">
         <v>34</v>
@@ -14520,7 +14520,7 @@
         <v>23</v>
       </c>
       <c r="K283" s="8">
-        <v>667</v>
+        <v>1020</v>
       </c>
       <c r="L283" s="9" t="s">
         <v>24</v>
@@ -14558,7 +14558,7 @@
         <v>23</v>
       </c>
       <c r="K284" s="13">
-        <v>241</v>
+        <v>532</v>
       </c>
       <c r="L284" s="15" t="s">
         <v>53</v>
@@ -14596,7 +14596,7 @@
         <v>23</v>
       </c>
       <c r="K285" s="8">
-        <v>778</v>
+        <v>243</v>
       </c>
       <c r="L285" s="9" t="s">
         <v>24</v>
@@ -14634,7 +14634,7 @@
         <v>23</v>
       </c>
       <c r="K286" s="13">
-        <v>1159</v>
+        <v>708</v>
       </c>
       <c r="L286" s="14" t="s">
         <v>34</v>
@@ -14672,7 +14672,7 @@
         <v>23</v>
       </c>
       <c r="K287" s="8">
-        <v>531</v>
+        <v>869</v>
       </c>
       <c r="L287" s="9" t="s">
         <v>24</v>
@@ -14710,7 +14710,7 @@
         <v>23</v>
       </c>
       <c r="K288" s="13">
-        <v>600</v>
+        <v>229</v>
       </c>
       <c r="L288" s="15" t="s">
         <v>53</v>
@@ -14748,7 +14748,7 @@
         <v>143</v>
       </c>
       <c r="K289" s="8">
-        <v>405</v>
+        <v>358</v>
       </c>
       <c r="L289" s="9" t="s">
         <v>24</v>
@@ -14786,7 +14786,7 @@
         <v>23</v>
       </c>
       <c r="K290" s="13">
-        <v>902</v>
+        <v>444</v>
       </c>
       <c r="L290" s="14" t="s">
         <v>34</v>
@@ -14824,7 +14824,7 @@
         <v>23</v>
       </c>
       <c r="K291" s="8">
-        <v>389</v>
+        <v>629</v>
       </c>
       <c r="L291" s="9" t="s">
         <v>24</v>
@@ -14862,7 +14862,7 @@
         <v>23</v>
       </c>
       <c r="K292" s="13">
-        <v>292</v>
+        <v>1042</v>
       </c>
       <c r="L292" s="16" t="s">
         <v>108</v>
@@ -14900,7 +14900,7 @@
         <v>23</v>
       </c>
       <c r="K293" s="8">
-        <v>1209</v>
+        <v>403</v>
       </c>
       <c r="L293" s="9" t="s">
         <v>24</v>
@@ -14938,7 +14938,7 @@
         <v>23</v>
       </c>
       <c r="K294" s="13">
-        <v>1057</v>
+        <v>1112</v>
       </c>
       <c r="L294" s="14" t="s">
         <v>34</v>
@@ -14976,7 +14976,7 @@
         <v>23</v>
       </c>
       <c r="K295" s="8">
-        <v>402</v>
+        <v>1035</v>
       </c>
       <c r="L295" s="9" t="s">
         <v>24</v>
@@ -15014,7 +15014,7 @@
         <v>23</v>
       </c>
       <c r="K296" s="13">
-        <v>1359</v>
+        <v>1230</v>
       </c>
       <c r="L296" s="15" t="s">
         <v>53</v>
@@ -15052,7 +15052,7 @@
         <v>23</v>
       </c>
       <c r="K297" s="8">
-        <v>873</v>
+        <v>954</v>
       </c>
       <c r="L297" s="9" t="s">
         <v>24</v>
@@ -15090,7 +15090,7 @@
         <v>23</v>
       </c>
       <c r="K298" s="13">
-        <v>244</v>
+        <v>1351</v>
       </c>
       <c r="L298" s="14" t="s">
         <v>34</v>
@@ -15128,7 +15128,7 @@
         <v>23</v>
       </c>
       <c r="K299" s="8">
-        <v>1300</v>
+        <v>786</v>
       </c>
       <c r="L299" s="9" t="s">
         <v>24</v>
@@ -15166,7 +15166,7 @@
         <v>23</v>
       </c>
       <c r="K300" s="13">
-        <v>769</v>
+        <v>842</v>
       </c>
       <c r="L300" s="15" t="s">
         <v>53</v>
@@ -15204,7 +15204,7 @@
         <v>23</v>
       </c>
       <c r="K301" s="8">
-        <v>833</v>
+        <v>454</v>
       </c>
       <c r="L301" s="9" t="s">
         <v>24</v>
@@ -15242,7 +15242,7 @@
         <v>23</v>
       </c>
       <c r="K302" s="13">
-        <v>929</v>
+        <v>991</v>
       </c>
       <c r="L302" s="14" t="s">
         <v>34</v>
@@ -15280,7 +15280,7 @@
         <v>23</v>
       </c>
       <c r="K303" s="8">
-        <v>357</v>
+        <v>451</v>
       </c>
       <c r="L303" s="9" t="s">
         <v>24</v>
@@ -15318,7 +15318,7 @@
         <v>23</v>
       </c>
       <c r="K304" s="13">
-        <v>528</v>
+        <v>817</v>
       </c>
       <c r="L304" s="16" t="s">
         <v>108</v>

</xml_diff>